<commit_message>
fix(hiv-template): format copies field
- add a comma separator to copies field

[Finishes ASP-1333]
</commit_message>
<xml_diff>
--- a/api/templates/results_hiv_not_suppressed/en.xlsx
+++ b/api/templates/results_hiv_not_suppressed/en.xlsx
@@ -83,10 +83,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -125,6 +126,13 @@
     </font>
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="16"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -214,18 +222,18 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="43" fontId="4" fillId="2" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="2" builtinId="3"/>

</xml_diff>

<commit_message>
Add caseId to reports and details screen, clean up details and reports a bit
</commit_message>
<xml_diff>
--- a/api/templates/results_hiv_not_suppressed/en.xlsx
+++ b/api/templates/results_hiv_not_suppressed/en.xlsx
@@ -1,10 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="22624"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A31DFE34-570F-4BEB-A6A9-7A6CC951CB2B}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6465"/>
+    <workbookView xWindow="45050" yWindow="1940" windowWidth="18040" windowHeight="15340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Results" sheetId="1" r:id="rId1"/>
@@ -14,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t>Patient ID</t>
   </si>
@@ -77,12 +78,18 @@
   </si>
   <si>
     <t>&lt;deviceName&gt;</t>
+  </si>
+  <si>
+    <t>Case ID</t>
+  </si>
+  <si>
+    <t>&lt;caseExternalId&gt;</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
@@ -238,7 +245,7 @@
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="2" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
@@ -296,7 +303,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -329,9 +336,26 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -364,6 +388,23 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -539,78 +580,83 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H8"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:I8"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="7.7109375" customWidth="1"/>
-    <col min="2" max="2" width="17.85546875" customWidth="1"/>
-    <col min="3" max="3" width="14.28515625" customWidth="1"/>
-    <col min="4" max="4" width="12.85546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="47.85546875" customWidth="1"/>
-    <col min="6" max="6" width="13.28515625" customWidth="1"/>
-    <col min="7" max="7" width="15.5703125" style="16" customWidth="1"/>
-    <col min="8" max="8" width="60.7109375" customWidth="1"/>
+    <col min="1" max="1" width="7.7265625" customWidth="1"/>
+    <col min="2" max="2" width="17.81640625" customWidth="1"/>
+    <col min="3" max="4" width="14.26953125" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="47.81640625" customWidth="1"/>
+    <col min="7" max="7" width="13.26953125" customWidth="1"/>
+    <col min="8" max="8" width="15.54296875" style="16" customWidth="1"/>
+    <col min="9" max="9" width="60.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.5">
       <c r="A1" s="2" t="s">
         <v>6</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="4"/>
       <c r="F1" s="2"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="2"/>
     </row>
-    <row r="2" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>14</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="3"/>
       <c r="F2" s="1"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="12"/>
+      <c r="I2" s="1"/>
     </row>
-    <row r="3" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>15</v>
       </c>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="3"/>
       <c r="F3" s="1"/>
-      <c r="G3" s="12"/>
-      <c r="H3" s="1"/>
+      <c r="G3" s="1"/>
+      <c r="H3" s="12"/>
+      <c r="I3" s="1"/>
     </row>
-    <row r="4" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>16</v>
       </c>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="3"/>
       <c r="F4" s="1"/>
-      <c r="G4" s="12"/>
-      <c r="H4" s="1"/>
+      <c r="G4" s="1"/>
+      <c r="H4" s="12"/>
+      <c r="I4" s="1"/>
     </row>
-    <row r="5" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="3"/>
       <c r="F5" s="1"/>
-      <c r="G5" s="12"/>
-      <c r="H5" s="1"/>
+      <c r="G5" s="1"/>
+      <c r="H5" s="12"/>
+      <c r="I5" s="1"/>
     </row>
-    <row r="6" spans="1:8" s="8" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" s="8" customFormat="1" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A6" s="7" t="s">
         <v>17</v>
       </c>
@@ -619,10 +665,11 @@
       <c r="D6" s="7"/>
       <c r="E6" s="7"/>
       <c r="F6" s="7"/>
-      <c r="G6" s="13"/>
-      <c r="H6" s="7"/>
+      <c r="G6" s="7"/>
+      <c r="H6" s="13"/>
+      <c r="I6" s="7"/>
     </row>
-    <row r="7" spans="1:8" s="5" customFormat="1" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" s="5" customFormat="1" ht="31" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="10" t="s">
         <v>2</v>
       </c>
@@ -633,22 +680,25 @@
         <v>1</v>
       </c>
       <c r="D7" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="E7" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="E7" s="10" t="s">
+      <c r="F7" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="F7" s="10" t="s">
+      <c r="G7" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="G7" s="14" t="s">
+      <c r="H7" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="H7" s="10" t="s">
+      <c r="I7" s="10" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A8" s="6" t="s">
         <v>18</v>
       </c>
@@ -659,18 +709,21 @@
         <v>10</v>
       </c>
       <c r="D8" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="E8" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="F8" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="G8" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="G8" s="15" t="s">
+      <c r="H8" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="H8" s="9" t="s">
+      <c r="I8" s="9" t="s">
         <v>13</v>
       </c>
     </row>

</xml_diff>